<commit_message>
Schematics and pins, 56 pins for ESP3-S3
</commit_message>
<xml_diff>
--- a/public/T-HMI_pins.xlsx
+++ b/public/T-HMI_pins.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="100">
   <si>
     <t>GPIO</t>
   </si>
@@ -25,24 +25,36 @@
     <t>S3 Pro</t>
   </si>
   <si>
+    <t>YD-ESP32-S3 N16R8</t>
+  </si>
+  <si>
     <t>BOOT</t>
   </si>
   <si>
     <t>Button</t>
   </si>
   <si>
+    <t>GPIO0</t>
+  </si>
+  <si>
     <t>LCD_SCLK</t>
   </si>
   <si>
     <t>A0</t>
   </si>
   <si>
+    <t>GPIO1</t>
+  </si>
+  <si>
     <t>LCD_CS</t>
   </si>
   <si>
     <t>A1</t>
   </si>
   <si>
+    <t>GPIO2</t>
+  </si>
+  <si>
     <t>LCD_MOSI</t>
   </si>
   <si>
@@ -52,30 +64,51 @@
     <t>Battery</t>
   </si>
   <si>
+    <t>GPIO3</t>
+  </si>
+  <si>
     <t>LCD_MISO</t>
   </si>
   <si>
     <t>A3</t>
   </si>
   <si>
+    <t>GPIO4</t>
+  </si>
+  <si>
+    <t>BATT_ADC</t>
+  </si>
+  <si>
     <t>A4</t>
   </si>
   <si>
+    <t>GPIO5</t>
+  </si>
+  <si>
     <t>A5</t>
   </si>
   <si>
+    <t>GPIO6</t>
+  </si>
+  <si>
     <t>LCD_DC</t>
   </si>
   <si>
     <t>A6</t>
   </si>
   <si>
+    <t>GPIO7</t>
+  </si>
+  <si>
     <t>LCD_PCLK</t>
   </si>
   <si>
     <t>A7</t>
   </si>
   <si>
+    <t>GPIO8</t>
+  </si>
+  <si>
     <t>LCD_IRQ</t>
   </si>
   <si>
@@ -85,6 +118,9 @@
     <t>SDA</t>
   </si>
   <si>
+    <t>GPIO9</t>
+  </si>
+  <si>
     <t>PWR_EN</t>
   </si>
   <si>
@@ -94,6 +130,9 @@
     <t>SCL</t>
   </si>
   <si>
+    <t>GPIO10</t>
+  </si>
+  <si>
     <t>SDIO_CMD</t>
   </si>
   <si>
@@ -103,6 +142,9 @@
     <t>MOSI</t>
   </si>
   <si>
+    <t>GPIO11</t>
+  </si>
+  <si>
     <t>SDIO_SCLK</t>
   </si>
   <si>
@@ -112,6 +154,9 @@
     <t>SCK</t>
   </si>
   <si>
+    <t>GPIO12</t>
+  </si>
+  <si>
     <t>SDIO_DATA0</t>
   </si>
   <si>
@@ -121,85 +166,151 @@
     <t>MISO</t>
   </si>
   <si>
+    <t>GPIO13</t>
+  </si>
+  <si>
     <t>PWR_ON</t>
   </si>
   <si>
     <t>TFT_LED</t>
   </si>
   <si>
+    <t>GPIO14</t>
+  </si>
+  <si>
     <t>Grove1</t>
   </si>
   <si>
     <t>A14</t>
   </si>
   <si>
+    <t>GPIO15</t>
+  </si>
+  <si>
     <t>A15</t>
   </si>
   <si>
+    <t>GPIO16</t>
+  </si>
+  <si>
     <t>Grove2</t>
   </si>
   <si>
     <t>A16</t>
   </si>
   <si>
+    <t>GPIO17</t>
+  </si>
+  <si>
     <t>A17</t>
   </si>
   <si>
+    <t>GPIO18</t>
+  </si>
+  <si>
     <t>Reed switch</t>
   </si>
   <si>
     <t>TFT_RST</t>
   </si>
   <si>
+    <t>GPIO21</t>
+  </si>
+  <si>
+    <t>nc</t>
+  </si>
+  <si>
+    <t>GPIO35</t>
+  </si>
+  <si>
+    <t>GPIO36</t>
+  </si>
+  <si>
+    <t>GPIO37</t>
+  </si>
+  <si>
     <t>LCD_BL</t>
   </si>
   <si>
     <t>RGB_LED</t>
   </si>
   <si>
+    <t>GPIO38</t>
+  </si>
+  <si>
     <t>LCD_DATA2</t>
   </si>
   <si>
+    <t>GPIO39</t>
+  </si>
+  <si>
     <t>LCD_DATA3</t>
   </si>
   <si>
+    <t>GPIO40</t>
+  </si>
+  <si>
     <t>LCD_DATA4</t>
   </si>
   <si>
+    <t>GPIO41</t>
+  </si>
+  <si>
     <t>LCD_DATA5</t>
   </si>
   <si>
+    <t>GPIO42</t>
+  </si>
+  <si>
     <t>Grove3</t>
   </si>
   <si>
     <t>TX0</t>
   </si>
   <si>
+    <t>GPIO43</t>
+  </si>
+  <si>
     <t>RX0</t>
   </si>
   <si>
+    <t>GPIO44</t>
+  </si>
+  <si>
     <t>LCD_DATA6</t>
   </si>
   <si>
     <t>TS_CS</t>
   </si>
   <si>
+    <t>GPIO45</t>
+  </si>
+  <si>
     <t>LCD_DATA7</t>
   </si>
   <si>
     <t>TF_CS</t>
   </si>
   <si>
+    <t>GPIO46</t>
+  </si>
+  <si>
     <t>LCD_DATA1</t>
   </si>
   <si>
     <t>TFT_DC</t>
   </si>
   <si>
+    <t>GPIO47</t>
+  </si>
+  <si>
     <t>LCD_DATA0</t>
   </si>
   <si>
     <t>TFT_CS</t>
+  </si>
+  <si>
+    <t>GPIO48</t>
   </si>
 </sst>
 </file>
@@ -239,12 +350,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -473,6 +587,7 @@
     <col customWidth="1" min="2" max="2" width="11.13"/>
     <col customWidth="1" min="3" max="3" width="5.88"/>
     <col customWidth="1" min="4" max="4" width="8.75"/>
+    <col customWidth="1" min="5" max="5" width="18.38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,388 +603,511 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>0.0</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>1.0</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>7</v>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>2.0</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>3.0</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>16</v>
+      <c r="C8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2">
+      <c r="A9" s="3">
         <v>7.0</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>18</v>
+      <c r="B9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>8.0</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>20</v>
+      <c r="B10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2">
+      <c r="A11" s="3">
         <v>9.0</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>23</v>
+      <c r="B11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2">
+      <c r="A12" s="3">
         <v>10.0</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>26</v>
+      <c r="B12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2">
+      <c r="A13" s="3">
         <v>11.0</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>29</v>
+      <c r="B13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2">
+      <c r="A14" s="3">
         <v>12.0</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>32</v>
+      <c r="B14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2">
+      <c r="A15" s="3">
         <v>13.0</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>35</v>
+      <c r="B15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2">
+      <c r="A16" s="3">
         <v>14.0</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="3">
+      <c r="B16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="4">
         <v>14.0</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>37</v>
+      <c r="D16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2">
+      <c r="A17" s="3">
         <v>15.0</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>39</v>
+      <c r="B17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2">
+      <c r="A18" s="3">
         <v>16.0</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>40</v>
+      <c r="B18" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2">
+      <c r="A19" s="3">
         <v>17.0</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>42</v>
+      <c r="B19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2">
+      <c r="A20" s="3">
         <v>18.0</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>43</v>
+      <c r="B20" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2">
+      <c r="A21" s="3">
         <v>21.0</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="3">
+      <c r="B21" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="4">
         <v>21.0</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>45</v>
+      <c r="D21" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2">
+      <c r="B22" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3">
         <v>38.0</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C22" s="3">
+      <c r="B25" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="4">
         <v>38.0</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2">
+      <c r="D25" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3">
         <v>39.0</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C23" s="3">
+      <c r="B26" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="4">
         <v>39.0</v>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2">
+      <c r="E26" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3">
         <v>40.0</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="3">
+      <c r="B27" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="4">
         <v>40.0</v>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2">
+      <c r="E27" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3">
         <v>41.0</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="3">
+      <c r="B28" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="4">
         <v>41.0</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2">
+      <c r="E28" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3">
         <v>42.0</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="3">
+      <c r="B29" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="4">
         <v>42.0</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2">
+      <c r="E29" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3">
         <v>43.0</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" s="3">
+      <c r="B30" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="4">
         <v>43.0</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2">
+      <c r="D30" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3">
         <v>44.0</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C28" s="3">
+      <c r="B31" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" s="4">
         <v>44.0</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2">
+      <c r="D31" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3">
         <v>45.0</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="3">
+      <c r="B32" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="4">
         <v>45.0</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2">
+      <c r="D32" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3">
         <v>46.0</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C30" s="3">
+      <c r="B33" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="4">
         <v>46.0</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2">
+      <c r="D33" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3">
         <v>47.0</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C31" s="3">
+      <c r="B34" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C34" s="4">
         <v>47.0</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2">
+      <c r="D34" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3">
         <v>48.0</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" s="3">
+      <c r="B35" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="4">
         <v>48.0</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>62</v>
+      <c r="D35" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>